<commit_message>
bug fixed: pre-existing file not loaded at start
</commit_message>
<xml_diff>
--- a/backup/rules_dynamic.xlsx
+++ b/backup/rules_dynamic.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="150">
   <si>
     <t>RuleSet</t>
   </si>
@@ -461,36 +461,6 @@
   </si>
   <si>
     <t>activeToFreeze3</t>
-  </si>
-  <si>
-    <t>activeToSuspend1</t>
-  </si>
-  <si>
-    <t>activeToSuspend</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>SUSPEND</t>
-  </si>
-  <si>
-    <t>activeToInactive1</t>
-  </si>
-  <si>
-    <t>activeToInactive</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>INACTIVE</t>
-  </si>
-  <si>
-    <t>sellingtoFreeze1</t>
-  </si>
-  <si>
-    <t>sellingToFreeze</t>
   </si>
 </sst>
 </file>
@@ -1808,7 +1778,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI18"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="28.6719" style="1" customWidth="1"/>
@@ -2909,362 +2879,41 @@
       </c>
     </row>
     <row r="15" ht="12.9" customHeight="1">
-      <c r="A15" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="B15" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="C15" t="s" s="20">
-        <v>142</v>
-      </c>
-      <c r="D15" t="s" s="20">
-        <v>152</v>
-      </c>
-      <c r="E15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="F15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="G15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="H15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="I15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="J15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="K15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="L15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="M15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="N15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="O15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="P15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Q15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="R15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="S15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="T15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="U15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="V15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="W15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="X15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Y15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Z15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AA15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AB15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AC15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AD15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AE15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AF15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AG15" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AH15" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI15" t="s" s="20">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="16" ht="12.9" customHeight="1">
-      <c r="A16" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="B16" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="C16" t="s" s="20">
-        <v>142</v>
-      </c>
-      <c r="D16" t="s" s="20">
-        <v>156</v>
-      </c>
-      <c r="E16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="F16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="G16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="H16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="I16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="J16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="K16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="L16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="M16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="N16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="O16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="P16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Q16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="R16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="S16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="T16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="U16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="V16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="W16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="X16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Y16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Z16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AA16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AB16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AC16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AD16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AE16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AF16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AG16" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AH16" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI16" t="s" s="20">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17" ht="12.9" customHeight="1">
-      <c r="A17" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="B17" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="C17" t="s" s="20">
-        <v>152</v>
-      </c>
-      <c r="D17" t="s" s="20">
-        <v>143</v>
-      </c>
-      <c r="E17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="F17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="G17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="H17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="I17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="J17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="K17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="L17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="M17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="N17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="O17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="P17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Q17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="R17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="S17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="T17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="U17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="V17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="W17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="X17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Y17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="Z17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AA17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AB17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AC17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AD17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AE17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AF17" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AG17" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AH17" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI17" t="s" s="20">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" ht="12.9" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
-      <c r="P18" s="20"/>
-      <c r="Q18" s="20"/>
-      <c r="R18" s="20"/>
-      <c r="S18" s="20"/>
-      <c r="T18" s="20"/>
-      <c r="U18" s="20"/>
-      <c r="V18" s="20"/>
-      <c r="W18" s="20"/>
-      <c r="X18" s="20"/>
-      <c r="Y18" s="20"/>
-      <c r="Z18" s="20"/>
-      <c r="AA18" s="20"/>
-      <c r="AB18" s="20"/>
-      <c r="AC18" s="20"/>
-      <c r="AD18" s="20"/>
-      <c r="AE18" s="20"/>
-      <c r="AF18" s="20"/>
-      <c r="AG18" s="20"/>
-      <c r="AH18" s="20"/>
-      <c r="AI18" s="20"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="20"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="20"/>
+      <c r="S15" s="20"/>
+      <c r="T15" s="20"/>
+      <c r="U15" s="20"/>
+      <c r="V15" s="20"/>
+      <c r="W15" s="20"/>
+      <c r="X15" s="20"/>
+      <c r="Y15" s="20"/>
+      <c r="Z15" s="20"/>
+      <c r="AA15" s="20"/>
+      <c r="AB15" s="20"/>
+      <c r="AC15" s="20"/>
+      <c r="AD15" s="20"/>
+      <c r="AE15" s="20"/>
+      <c r="AF15" s="20"/>
+      <c r="AG15" s="20"/>
+      <c r="AH15" s="20"/>
+      <c r="AI15" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>